<commit_message>
Tax Zeigelei as Hofraum
</commit_message>
<xml_diff>
--- a/kulturarten.xlsx
+++ b/kulturarten.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE066280-7B83-45EC-959D-344B60AF71BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE89D97-3470-4DF6-88EC-023C3C085944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3771" yWindow="1491" windowWidth="17375" windowHeight="16303" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="191">
   <si>
     <t>Kulturart</t>
   </si>
@@ -1646,6 +1646,9 @@
       <c r="B67" t="s">
         <v>67</v>
       </c>
+      <c r="C67" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A68" t="s">

</xml_diff>

<commit_message>
Tax heide as heide for gemeinde clarholz
</commit_message>
<xml_diff>
--- a/kulturarten.xlsx
+++ b/kulturarten.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE89D97-3470-4DF6-88EC-023C3C085944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8723593-1F8A-464F-BE0E-ECAEB360064F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="192">
   <si>
     <t>Kulturart</t>
   </si>
@@ -593,6 +593,9 @@
   </si>
   <si>
     <t>haus ohne grund</t>
+  </si>
+  <si>
+    <t>Hütung;Clarholz=Heide</t>
   </si>
 </sst>
 </file>
@@ -1817,7 +1820,7 @@
         <v>82</v>
       </c>
       <c r="C86" t="s">
-        <v>159</v>
+        <v>191</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Tax lache as öde
</commit_message>
<xml_diff>
--- a/kulturarten.xlsx
+++ b/kulturarten.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8723593-1F8A-464F-BE0E-ECAEB360064F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE117BF5-79E2-4B17-A4EE-9A68CE78C3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="193">
   <si>
     <t>Kulturart</t>
   </si>
@@ -596,6 +596,9 @@
   </si>
   <si>
     <t>Hütung;Clarholz=Heide</t>
+  </si>
+  <si>
+    <t>Öde</t>
   </si>
 </sst>
 </file>
@@ -1110,7 +1113,7 @@
         <v>161</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">

</xml_diff>